<commit_message>
Update talk details and add new talk on green waste management
</commit_message>
<xml_diff>
--- a/markdown_generator/talks.xlsx
+++ b/markdown_generator/talks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10469826_polimi_it/Documents/Dottorato/Curriculum/Nick-Bertoldo.github.io/markdown_generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="11_F25DC773A252ABDACC10486189DB5B345BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E2B407D-7926-4CFD-87DD-862A42AC889C}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="11_F25DC773A252ABDACC10486189DB5B345BDE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3144DD0F-3DB7-43AF-AE6E-E51E58C1C75E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
   <si>
     <t>title</t>
   </si>
@@ -78,9 +78,6 @@
     <t>The potential environmental benefit of the ecodesign approach: a case study in the footwear industry</t>
   </si>
   <si>
-    <t>XVI conference of the Associazione Rete Italiana LCA</t>
-  </si>
-  <si>
     <t>RILCA23</t>
   </si>
   <si>
@@ -91,6 +88,27 @@
   </si>
   <si>
     <t>This work explores the application of ecodesign principles within the footwear industry by integrating Life Cycle Assessment (LCA). We modeled 21 materials and compared traditional footwear designs with alternatives developed using specific ecodesign principles. The results demonstrate that these ecodesign-driven material choices generally lead to reduced environmental impacts across various categories.</t>
+  </si>
+  <si>
+    <t>Life Cycle Assessment of Green Waste Management: Optimizing Composting Facility Distribution in the Milan Metropolitan Area</t>
+  </si>
+  <si>
+    <t>RILCA25</t>
+  </si>
+  <si>
+    <t>XIX conference of the Associazione Rete Italiana LCA</t>
+  </si>
+  <si>
+    <t>XVII conference of the Associazione Rete Italiana LCA</t>
+  </si>
+  <si>
+    <t>19-03-2025</t>
+  </si>
+  <si>
+    <t>Cortina d'Ampezzo</t>
+  </si>
+  <si>
+    <t>The disposal of garden waste from green space maintenance (dry leaves, pruning and brushwood) represents not only a cost for public authorities but also an environmental impact in terms of transportation. This study analyses the impact of different location choices of garden waste composting plants using the case study of the Metropolitan City of Milan. The current reference scenario is compared to an ideal scenario with a more equal distribution of composting capacity in the metropolitan area. These scenarios are then compared through a Life Cycle Assessment study, to evaluate their environmental performances. Optimizing composting plant locations could reduce the environmental impacts of green waste management, especially by reducing transport distances. These findings emphasize the importance of distributing green waste plants and the potential for utilizing the obtained compost within urban green spaces.</t>
   </si>
 </sst>
 </file>
@@ -135,10 +153,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -420,8 +440,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="5" max="5" width="10.5546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -450,57 +473,80 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>8</v>
+      <c r="A2" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>15</v>
+        <v>23</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="H2" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
       </c>
       <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="1" t="s">
+      <c r="F4" t="s">
         <v>19</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H4" t="s">
         <v>20</v>
-      </c>
-      <c r="H3" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{E76240B0-155A-459B-B621-19BF871C9664}"/>
+    <hyperlink ref="G3" r:id="rId1" xr:uid="{E76240B0-155A-459B-B621-19BF871C9664}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>